<commit_message>
Added task 4 data and code
</commit_message>
<xml_diff>
--- a/Practical3/STM32F0_Task3_Data.xlsx
+++ b/Practical3/STM32F0_Task3_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/ngrmar007_myuct_ac_za/Documents/Third Year/EEE3096s-repository/EEE3096S-Group-39/Practical3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{CD99EA7B-D802-48B2-B751-A2CA09ED7869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A03BCC78-63DD-4058-AEE3-FACE47D7F7B4}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{CD99EA7B-D802-48B2-B751-A2CA09ED7869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7223CA8-67E9-46A4-8AF6-C169CDE426F6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7F0029D-43E0-4630-A09B-07C2D8494090}"/>
+    <workbookView xWindow="-336" yWindow="1092" windowWidth="10896" windowHeight="10008" xr2:uid="{B7F0029D-43E0-4630-A09B-07C2D8494090}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Image Size</t>
   </si>
@@ -53,22 +53,19 @@
     <t>Clock Cycles</t>
   </si>
   <si>
-    <t>18446744073639093271'</t>
-  </si>
-  <si>
-    <t>1663030774'</t>
-  </si>
-  <si>
-    <t>1054369028'</t>
-  </si>
-  <si>
-    <t>18446744072682874475'</t>
-  </si>
-  <si>
-    <t>18446744071810763853'</t>
-  </si>
-  <si>
-    <t>*</t>
+    <t>1054369040'</t>
+  </si>
+  <si>
+    <t>1663030772'</t>
+  </si>
+  <si>
+    <t>2396179548'</t>
+  </si>
+  <si>
+    <t>3268290164'</t>
+  </si>
+  <si>
+    <t>4224508960'</t>
   </si>
 </sst>
 </file>
@@ -127,6 +124,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -446,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{403677A3-D7C6-4BA9-86A2-ED163CC34853}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.44140625" style="1" customWidth="1"/>
@@ -456,7 +457,7 @@
     <col min="5" max="5" width="27" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -473,7 +474,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>128</v>
       </c>
@@ -487,10 +488,10 @@
         <v>745</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>160</v>
       </c>
@@ -507,7 +508,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>192</v>
       </c>
@@ -521,13 +522,10 @@
         <v>738</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>224</v>
       </c>
@@ -543,11 +541,8 @@
       <c r="E5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>256</v>
       </c>
@@ -561,10 +556,7 @@
         <v>744</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>